<commit_message>
update of flodym material - 4 of 5 workbooks complete.
</commit_message>
<xml_diff>
--- a/2_focus_groups/23_flodym_deepdive_Stefan_Pauliuk/input_data/example5_eol_recovery_rate.xlsx
+++ b/2_focus_groups/23_flodym_deepdive_Stefan_Pauliuk/input_data/example5_eol_recovery_rate.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867C4319-4D92-4F01-911F-F6A6E8A8BC15}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA63D9D-F906-4D62-A251-49E4FE048097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="6450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="3" r:id="rId1"/>
     <sheet name="Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -468,7 +473,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -484,9 +489,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -524,9 +529,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -559,26 +564,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -611,26 +599,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -805,15 +776,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.90625" customWidth="1"/>
-    <col min="3" max="3" width="19.1796875" customWidth="1"/>
-    <col min="4" max="4" width="31.453125" customWidth="1"/>
+    <col min="1" max="1" width="34.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" customWidth="1"/>
+    <col min="4" max="4" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>41</v>
       </c>
@@ -824,7 +795,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -838,7 +809,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>19</v>
       </c>
@@ -852,7 +823,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>21</v>
       </c>
@@ -866,7 +837,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>1</v>
       </c>
@@ -880,7 +851,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>5</v>
       </c>
@@ -894,7 +865,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>6</v>
       </c>
@@ -908,7 +879,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
@@ -922,7 +893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>25</v>
       </c>
@@ -936,7 +907,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>26</v>
       </c>
@@ -950,7 +921,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>28</v>
       </c>
@@ -964,7 +935,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>30</v>
       </c>
@@ -978,7 +949,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>32</v>
       </c>
@@ -992,7 +963,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>35</v>
       </c>
@@ -1006,7 +977,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>37</v>
       </c>
@@ -1020,7 +991,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>48</v>
       </c>
@@ -1028,7 +999,7 @@
       <c r="C16" s="5"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>48</v>
       </c>
@@ -1036,7 +1007,7 @@
       <c r="C17" s="5"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>48</v>
       </c>
@@ -1044,7 +1015,7 @@
       <c r="C18" s="5"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>48</v>
       </c>
@@ -1052,7 +1023,7 @@
       <c r="C19" s="5"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>48</v>
       </c>
@@ -1060,7 +1031,7 @@
       <c r="C20" s="5"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>2</v>
       </c>
@@ -1080,7 +1051,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>10</v>
       </c>
@@ -1100,7 +1071,7 @@
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="18" t="s">
         <v>61</v>
       </c>
@@ -1122,7 +1093,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
         <v>68</v>
       </c>
@@ -1144,7 +1115,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
         <v>69</v>
       </c>
@@ -1166,7 +1137,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C26" s="18" t="s">
         <v>14</v>
       </c>
@@ -1182,7 +1153,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C27" s="18" t="s">
         <v>15</v>
       </c>
@@ -1195,7 +1166,7 @@
       <c r="F27" s="5"/>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E28" s="1" t="s">
         <v>16</v>
       </c>
@@ -1210,21 +1181,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:T421"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.36328125" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="3" max="3" width="24.90625" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" customWidth="1"/>
-    <col min="9" max="9" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>50</v>
       </c>
@@ -1250,7 +1221,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -1277,7 +1248,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -1304,7 +1275,7 @@
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1331,7 +1302,7 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>62</v>
       </c>
@@ -1358,7 +1329,7 @@
       </c>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>62</v>
       </c>
@@ -1385,7 +1356,7 @@
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>62</v>
       </c>
@@ -1412,7 +1383,7 @@
       </c>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -1439,7 +1410,7 @@
       </c>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -1466,7 +1437,7 @@
       </c>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -1493,7 +1464,7 @@
       </c>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -1520,7 +1491,7 @@
       </c>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>62</v>
       </c>
@@ -1547,7 +1518,7 @@
       </c>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -1574,7 +1545,7 @@
       </c>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>62</v>
       </c>
@@ -1601,7 +1572,7 @@
       </c>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -1628,7 +1599,7 @@
       </c>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>62</v>
       </c>
@@ -1655,7 +1626,7 @@
       </c>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>62</v>
       </c>
@@ -1684,7 +1655,7 @@
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>62</v>
       </c>
@@ -1713,7 +1684,7 @@
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -1742,7 +1713,7 @@
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -1771,7 +1742,7 @@
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>62</v>
       </c>
@@ -1800,7 +1771,7 @@
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>62</v>
       </c>
@@ -1829,7 +1800,7 @@
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -1858,7 +1829,7 @@
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -1887,7 +1858,7 @@
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -1916,7 +1887,7 @@
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>62</v>
       </c>
@@ -1945,1665 +1916,1665 @@
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="T27" s="4"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
       <c r="T28" s="4"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
       <c r="T29" s="4"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="T30" s="4"/>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
       <c r="T31" s="4"/>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
       <c r="T32" s="4"/>
     </row>
-    <row r="33" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="33" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
       <c r="T33" s="4"/>
     </row>
-    <row r="34" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="34" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="T34" s="4"/>
     </row>
-    <row r="35" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="35" spans="5:20" x14ac:dyDescent="0.3">
       <c r="E35" s="1"/>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="T35" s="4"/>
     </row>
-    <row r="36" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="36" spans="5:20" x14ac:dyDescent="0.3">
       <c r="E36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="T36" s="4"/>
     </row>
-    <row r="37" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="37" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
       <c r="T37" s="4"/>
     </row>
-    <row r="38" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="38" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
       <c r="T38" s="4"/>
     </row>
-    <row r="39" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="39" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="T39" s="4"/>
     </row>
-    <row r="40" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="40" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="T40" s="4"/>
     </row>
-    <row r="41" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="41" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="T41" s="4"/>
     </row>
-    <row r="42" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="42" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
     </row>
-    <row r="43" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="43" spans="5:20" x14ac:dyDescent="0.3">
       <c r="G43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
     </row>
-    <row r="44" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="44" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
     </row>
-    <row r="45" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="45" spans="5:20" x14ac:dyDescent="0.3">
       <c r="G45" s="4"/>
       <c r="I45" s="4"/>
       <c r="J45" s="4"/>
     </row>
-    <row r="46" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="46" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
     </row>
-    <row r="47" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="47" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I47" s="4"/>
       <c r="J47" s="4"/>
     </row>
-    <row r="48" spans="5:20" x14ac:dyDescent="0.35">
+    <row r="48" spans="5:20" x14ac:dyDescent="0.3">
       <c r="I48" s="4"/>
       <c r="J48" s="4"/>
     </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I49" s="4"/>
       <c r="J49" s="4"/>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I50" s="4"/>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B52" s="4"/>
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
     </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B53" s="4"/>
       <c r="I53" s="4"/>
       <c r="J53" s="4"/>
     </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B54" s="4"/>
       <c r="I54" s="4"/>
       <c r="J54" s="4"/>
     </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B55" s="4"/>
       <c r="I55" s="4"/>
       <c r="J55" s="4"/>
     </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
     </row>
-    <row r="57" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B57" s="4"/>
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
     </row>
-    <row r="58" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B58" s="4"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4"/>
     </row>
-    <row r="59" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B59" s="4"/>
       <c r="I59" s="4"/>
       <c r="J59" s="4"/>
     </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B60" s="4"/>
       <c r="I60" s="4"/>
       <c r="J60" s="4"/>
     </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="4"/>
     </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B62" s="4"/>
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
     </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B63" s="4"/>
       <c r="I63" s="4"/>
       <c r="J63" s="4"/>
     </row>
-    <row r="64" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B64" s="4"/>
       <c r="I64" s="4"/>
       <c r="J64" s="4"/>
     </row>
-    <row r="65" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B65" s="4"/>
       <c r="I65" s="4"/>
       <c r="J65" s="4"/>
     </row>
-    <row r="69" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:10" x14ac:dyDescent="0.3">
       <c r="G69" s="4"/>
     </row>
-    <row r="82" spans="7:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G82" s="4"/>
     </row>
-    <row r="98" spans="7:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G98" s="4"/>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
       <c r="C132" s="4"/>
       <c r="D132" s="4"/>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="4"/>
       <c r="C133" s="4"/>
       <c r="D133" s="4"/>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="4"/>
       <c r="C134" s="4"/>
       <c r="D134" s="4"/>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="4"/>
       <c r="C135" s="4"/>
       <c r="D135" s="4"/>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="4"/>
       <c r="C136" s="4"/>
       <c r="D136" s="4"/>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="4"/>
       <c r="C137" s="4"/>
       <c r="D137" s="4"/>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="4"/>
       <c r="C138" s="4"/>
       <c r="D138" s="4"/>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="4"/>
       <c r="C139" s="4"/>
       <c r="D139" s="4"/>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" s="4"/>
       <c r="C140" s="4"/>
       <c r="D140" s="4"/>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" s="4"/>
       <c r="C141" s="4"/>
       <c r="D141" s="4"/>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" s="4"/>
       <c r="C142" s="4"/>
       <c r="D142" s="4"/>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="4"/>
       <c r="C143" s="4"/>
       <c r="D143" s="4"/>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" s="4"/>
       <c r="C144" s="4"/>
       <c r="D144" s="4"/>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" s="4"/>
       <c r="C145" s="4"/>
       <c r="D145" s="4"/>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" s="4"/>
       <c r="C146" s="4"/>
       <c r="D146" s="4"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="4"/>
       <c r="C147" s="4"/>
       <c r="D147" s="4"/>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="4"/>
       <c r="C148" s="4"/>
       <c r="D148" s="4"/>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
       <c r="C149" s="4"/>
       <c r="D149" s="4"/>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" s="4"/>
       <c r="C150" s="4"/>
       <c r="D150" s="4"/>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" s="4"/>
       <c r="C151" s="4"/>
       <c r="D151" s="4"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" s="4"/>
       <c r="C152" s="4"/>
       <c r="D152" s="4"/>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" s="4"/>
       <c r="C153" s="4"/>
       <c r="D153" s="4"/>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" s="4"/>
       <c r="C154" s="4"/>
       <c r="D154" s="4"/>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" s="4"/>
       <c r="C155" s="4"/>
       <c r="D155" s="4"/>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" s="4"/>
       <c r="C156" s="4"/>
       <c r="D156" s="4"/>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" s="4"/>
       <c r="C157" s="4"/>
       <c r="D157" s="4"/>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" s="4"/>
       <c r="C158" s="4"/>
       <c r="D158" s="4"/>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" s="4"/>
       <c r="C159" s="4"/>
       <c r="D159" s="4"/>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" s="4"/>
       <c r="C160" s="4"/>
       <c r="D160" s="4"/>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="4"/>
       <c r="C161" s="4"/>
       <c r="D161" s="4"/>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="4"/>
       <c r="C162" s="4"/>
       <c r="D162" s="4"/>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" s="4"/>
       <c r="C163" s="4"/>
       <c r="D163" s="4"/>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" s="4"/>
       <c r="C164" s="4"/>
       <c r="D164" s="4"/>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" s="4"/>
       <c r="C165" s="4"/>
       <c r="D165" s="4"/>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" s="4"/>
       <c r="C166" s="4"/>
       <c r="D166" s="4"/>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" s="4"/>
       <c r="C167" s="4"/>
       <c r="D167" s="4"/>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" s="4"/>
       <c r="C168" s="4"/>
       <c r="D168" s="4"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" s="4"/>
       <c r="C169" s="4"/>
       <c r="D169" s="4"/>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" s="4"/>
       <c r="C170" s="4"/>
       <c r="D170" s="4"/>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" s="4"/>
       <c r="C171" s="4"/>
       <c r="D171" s="4"/>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172" s="4"/>
       <c r="C172" s="4"/>
       <c r="D172" s="4"/>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" s="4"/>
       <c r="C173" s="4"/>
       <c r="D173" s="4"/>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174" s="4"/>
       <c r="C174" s="4"/>
       <c r="D174" s="4"/>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175" s="4"/>
       <c r="C175" s="4"/>
       <c r="D175" s="4"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A176" s="4"/>
       <c r="C176" s="4"/>
       <c r="D176" s="4"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A177" s="4"/>
       <c r="C177" s="4"/>
       <c r="D177" s="4"/>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A178" s="4"/>
       <c r="C178" s="4"/>
       <c r="D178" s="4"/>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A179" s="4"/>
       <c r="C179" s="4"/>
       <c r="D179" s="4"/>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A180" s="4"/>
       <c r="C180" s="4"/>
       <c r="D180" s="4"/>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A181" s="4"/>
       <c r="C181" s="4"/>
       <c r="D181" s="4"/>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A182" s="4"/>
       <c r="C182" s="4"/>
       <c r="D182" s="4"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A183" s="4"/>
       <c r="C183" s="4"/>
       <c r="D183" s="4"/>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A184" s="4"/>
       <c r="C184" s="4"/>
       <c r="D184" s="4"/>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A185" s="4"/>
       <c r="C185" s="4"/>
       <c r="D185" s="4"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A186" s="4"/>
       <c r="C186" s="4"/>
       <c r="D186" s="4"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A187" s="4"/>
       <c r="C187" s="4"/>
       <c r="D187" s="4"/>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A188" s="4"/>
       <c r="C188" s="4"/>
       <c r="D188" s="4"/>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A189" s="4"/>
       <c r="C189" s="4"/>
       <c r="D189" s="4"/>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A190" s="4"/>
       <c r="C190" s="4"/>
       <c r="D190" s="4"/>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A191" s="4"/>
       <c r="C191" s="4"/>
       <c r="D191" s="4"/>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A192" s="4"/>
       <c r="C192" s="4"/>
       <c r="D192" s="4"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A193" s="4"/>
       <c r="C193" s="4"/>
       <c r="D193" s="4"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A194" s="4"/>
       <c r="C194" s="4"/>
       <c r="D194" s="4"/>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A195" s="4"/>
       <c r="C195" s="4"/>
       <c r="D195" s="4"/>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A196" s="4"/>
       <c r="C196" s="4"/>
       <c r="D196" s="4"/>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A197" s="4"/>
       <c r="C197" s="4"/>
       <c r="D197" s="4"/>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A198" s="4"/>
       <c r="C198" s="4"/>
       <c r="D198" s="4"/>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A199" s="4"/>
       <c r="C199" s="4"/>
       <c r="D199" s="4"/>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A200" s="4"/>
       <c r="C200" s="4"/>
       <c r="D200" s="4"/>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A201" s="4"/>
       <c r="C201" s="4"/>
       <c r="D201" s="4"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A202" s="4"/>
       <c r="C202" s="4"/>
       <c r="D202" s="4"/>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A203" s="4"/>
       <c r="C203" s="4"/>
       <c r="D203" s="4"/>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A204" s="4"/>
       <c r="C204" s="4"/>
       <c r="D204" s="4"/>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A205" s="4"/>
       <c r="C205" s="4"/>
       <c r="D205" s="4"/>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A206" s="4"/>
       <c r="C206" s="4"/>
       <c r="D206" s="4"/>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A207" s="4"/>
       <c r="C207" s="4"/>
       <c r="D207" s="4"/>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A208" s="4"/>
       <c r="C208" s="4"/>
       <c r="D208" s="4"/>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A209" s="4"/>
       <c r="C209" s="4"/>
       <c r="D209" s="4"/>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A210" s="4"/>
       <c r="C210" s="4"/>
       <c r="D210" s="4"/>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A211" s="4"/>
       <c r="C211" s="4"/>
       <c r="D211" s="4"/>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A212" s="4"/>
       <c r="C212" s="4"/>
       <c r="D212" s="4"/>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A213" s="4"/>
       <c r="C213" s="4"/>
       <c r="D213" s="4"/>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A214" s="4"/>
       <c r="C214" s="4"/>
       <c r="D214" s="4"/>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A215" s="4"/>
       <c r="C215" s="4"/>
       <c r="D215" s="4"/>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A216" s="4"/>
       <c r="C216" s="4"/>
       <c r="D216" s="4"/>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A217" s="4"/>
       <c r="C217" s="4"/>
       <c r="D217" s="4"/>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A218" s="4"/>
       <c r="C218" s="4"/>
       <c r="D218" s="4"/>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A219" s="4"/>
       <c r="C219" s="4"/>
       <c r="D219" s="4"/>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A220" s="4"/>
       <c r="C220" s="4"/>
       <c r="D220" s="4"/>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A221" s="4"/>
       <c r="C221" s="4"/>
       <c r="D221" s="4"/>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A222" s="4"/>
       <c r="C222" s="4"/>
       <c r="D222" s="4"/>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A223" s="4"/>
       <c r="C223" s="4"/>
       <c r="D223" s="4"/>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A224" s="4"/>
       <c r="C224" s="4"/>
       <c r="D224" s="4"/>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A225" s="4"/>
       <c r="C225" s="4"/>
       <c r="D225" s="4"/>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A226" s="4"/>
       <c r="C226" s="4"/>
       <c r="D226" s="4"/>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A227" s="4"/>
       <c r="C227" s="4"/>
       <c r="D227" s="4"/>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A228" s="4"/>
       <c r="C228" s="4"/>
       <c r="D228" s="4"/>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A229" s="4"/>
       <c r="C229" s="4"/>
       <c r="D229" s="4"/>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A230" s="4"/>
       <c r="C230" s="4"/>
       <c r="D230" s="4"/>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A231" s="4"/>
       <c r="C231" s="4"/>
       <c r="D231" s="4"/>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A232" s="4"/>
       <c r="C232" s="4"/>
       <c r="D232" s="4"/>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A233" s="4"/>
       <c r="C233" s="4"/>
       <c r="D233" s="4"/>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A234" s="4"/>
       <c r="C234" s="4"/>
       <c r="D234" s="4"/>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A235" s="4"/>
       <c r="C235" s="4"/>
       <c r="D235" s="4"/>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A236" s="4"/>
       <c r="C236" s="4"/>
       <c r="D236" s="4"/>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A237" s="4"/>
       <c r="C237" s="4"/>
       <c r="D237" s="4"/>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A238" s="4"/>
       <c r="C238" s="4"/>
       <c r="D238" s="4"/>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A239" s="4"/>
       <c r="C239" s="4"/>
       <c r="D239" s="4"/>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A240" s="4"/>
       <c r="C240" s="4"/>
       <c r="D240" s="4"/>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A241" s="4"/>
       <c r="C241" s="4"/>
       <c r="D241" s="4"/>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A242" s="4"/>
       <c r="C242" s="4"/>
       <c r="D242" s="4"/>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A243" s="4"/>
       <c r="C243" s="4"/>
       <c r="D243" s="4"/>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A244" s="4"/>
       <c r="C244" s="4"/>
       <c r="D244" s="4"/>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A245" s="4"/>
       <c r="C245" s="4"/>
       <c r="D245" s="4"/>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A246" s="4"/>
       <c r="C246" s="4"/>
       <c r="D246" s="4"/>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A247" s="4"/>
       <c r="C247" s="4"/>
       <c r="D247" s="4"/>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A248" s="4"/>
       <c r="C248" s="4"/>
       <c r="D248" s="4"/>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A249" s="4"/>
       <c r="C249" s="4"/>
       <c r="D249" s="4"/>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A250" s="4"/>
       <c r="C250" s="4"/>
       <c r="D250" s="4"/>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A251" s="4"/>
       <c r="C251" s="4"/>
       <c r="D251" s="4"/>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A252" s="4"/>
       <c r="C252" s="4"/>
       <c r="D252" s="4"/>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A253" s="4"/>
       <c r="C253" s="4"/>
       <c r="D253" s="4"/>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A254" s="4"/>
       <c r="C254" s="4"/>
       <c r="D254" s="4"/>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A255" s="4"/>
       <c r="C255" s="4"/>
       <c r="D255" s="4"/>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A256" s="4"/>
       <c r="C256" s="4"/>
       <c r="D256" s="4"/>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A257" s="4"/>
       <c r="C257" s="4"/>
       <c r="D257" s="4"/>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A258" s="4"/>
       <c r="C258" s="4"/>
       <c r="D258" s="4"/>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A259" s="4"/>
       <c r="C259" s="4"/>
       <c r="D259" s="4"/>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A260" s="4"/>
       <c r="C260" s="4"/>
       <c r="D260" s="4"/>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A261" s="4"/>
       <c r="C261" s="4"/>
       <c r="D261" s="4"/>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A262" s="4"/>
       <c r="C262" s="4"/>
       <c r="D262" s="4"/>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A263" s="4"/>
       <c r="C263" s="4"/>
       <c r="D263" s="4"/>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A264" s="4"/>
       <c r="C264" s="4"/>
       <c r="D264" s="4"/>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A265" s="4"/>
       <c r="C265" s="4"/>
       <c r="D265" s="4"/>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A266" s="4"/>
       <c r="C266" s="4"/>
       <c r="D266" s="4"/>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A267" s="4"/>
       <c r="C267" s="4"/>
       <c r="D267" s="4"/>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A268" s="4"/>
       <c r="C268" s="4"/>
       <c r="D268" s="4"/>
     </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A269" s="4"/>
       <c r="C269" s="4"/>
       <c r="D269" s="4"/>
     </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A270" s="4"/>
       <c r="C270" s="4"/>
       <c r="D270" s="4"/>
     </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A271" s="4"/>
       <c r="C271" s="4"/>
       <c r="D271" s="4"/>
     </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A272" s="4"/>
       <c r="C272" s="4"/>
       <c r="D272" s="4"/>
     </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A273" s="4"/>
       <c r="C273" s="4"/>
       <c r="D273" s="4"/>
     </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A274" s="4"/>
       <c r="C274" s="4"/>
       <c r="D274" s="4"/>
     </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A275" s="4"/>
       <c r="C275" s="4"/>
       <c r="D275" s="4"/>
     </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A276" s="4"/>
       <c r="C276" s="4"/>
       <c r="D276" s="4"/>
     </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A277" s="4"/>
       <c r="C277" s="4"/>
       <c r="D277" s="4"/>
     </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A278" s="4"/>
       <c r="C278" s="4"/>
       <c r="D278" s="4"/>
     </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A279" s="4"/>
       <c r="C279" s="4"/>
       <c r="D279" s="4"/>
     </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A280" s="4"/>
       <c r="C280" s="4"/>
       <c r="D280" s="4"/>
     </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A281" s="4"/>
       <c r="C281" s="4"/>
       <c r="D281" s="4"/>
     </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A282" s="4"/>
       <c r="C282" s="4"/>
       <c r="D282" s="4"/>
     </row>
-    <row r="283" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A283" s="4"/>
       <c r="C283" s="4"/>
       <c r="D283" s="4"/>
     </row>
-    <row r="284" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A284" s="4"/>
       <c r="C284" s="4"/>
       <c r="D284" s="4"/>
     </row>
-    <row r="285" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A285" s="4"/>
       <c r="C285" s="4"/>
       <c r="D285" s="4"/>
     </row>
-    <row r="286" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A286" s="4"/>
       <c r="C286" s="4"/>
       <c r="D286" s="4"/>
     </row>
-    <row r="287" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A287" s="4"/>
       <c r="C287" s="4"/>
       <c r="D287" s="4"/>
     </row>
-    <row r="288" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A288" s="4"/>
       <c r="C288" s="4"/>
       <c r="D288" s="4"/>
     </row>
-    <row r="289" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A289" s="4"/>
       <c r="C289" s="4"/>
       <c r="D289" s="4"/>
     </row>
-    <row r="290" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A290" s="4"/>
       <c r="C290" s="4"/>
       <c r="D290" s="4"/>
     </row>
-    <row r="291" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A291" s="4"/>
       <c r="C291" s="4"/>
       <c r="D291" s="4"/>
     </row>
-    <row r="292" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A292" s="4"/>
       <c r="C292" s="4"/>
       <c r="D292" s="4"/>
     </row>
-    <row r="293" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A293" s="4"/>
       <c r="C293" s="4"/>
       <c r="D293" s="4"/>
     </row>
-    <row r="294" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A294" s="4"/>
       <c r="C294" s="4"/>
       <c r="D294" s="4"/>
     </row>
-    <row r="295" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A295" s="4"/>
       <c r="C295" s="4"/>
       <c r="D295" s="4"/>
     </row>
-    <row r="296" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A296" s="4"/>
       <c r="C296" s="4"/>
       <c r="D296" s="4"/>
     </row>
-    <row r="297" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A297" s="4"/>
       <c r="C297" s="4"/>
       <c r="D297" s="4"/>
     </row>
-    <row r="298" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A298" s="4"/>
       <c r="C298" s="4"/>
       <c r="D298" s="4"/>
     </row>
-    <row r="299" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A299" s="4"/>
       <c r="C299" s="4"/>
       <c r="D299" s="4"/>
     </row>
-    <row r="300" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A300" s="4"/>
       <c r="C300" s="4"/>
       <c r="D300" s="4"/>
     </row>
-    <row r="301" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A301" s="4"/>
       <c r="C301" s="4"/>
       <c r="D301" s="4"/>
     </row>
-    <row r="302" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A302" s="4"/>
       <c r="C302" s="4"/>
       <c r="D302" s="4"/>
     </row>
-    <row r="303" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A303" s="4"/>
       <c r="C303" s="4"/>
       <c r="D303" s="4"/>
     </row>
-    <row r="304" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A304" s="4"/>
       <c r="C304" s="4"/>
       <c r="D304" s="4"/>
     </row>
-    <row r="305" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A305" s="4"/>
       <c r="C305" s="4"/>
       <c r="D305" s="4"/>
     </row>
-    <row r="306" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A306" s="4"/>
       <c r="C306" s="4"/>
       <c r="D306" s="4"/>
     </row>
-    <row r="307" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A307" s="4"/>
       <c r="C307" s="4"/>
       <c r="D307" s="4"/>
     </row>
-    <row r="308" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A308" s="4"/>
       <c r="C308" s="4"/>
       <c r="D308" s="4"/>
     </row>
-    <row r="309" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A309" s="4"/>
       <c r="C309" s="4"/>
       <c r="D309" s="4"/>
     </row>
-    <row r="310" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A310" s="4"/>
       <c r="C310" s="4"/>
       <c r="D310" s="4"/>
     </row>
-    <row r="311" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A311" s="4"/>
       <c r="C311" s="4"/>
       <c r="D311" s="4"/>
     </row>
-    <row r="312" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A312" s="4"/>
       <c r="C312" s="4"/>
       <c r="D312" s="4"/>
     </row>
-    <row r="313" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A313" s="4"/>
       <c r="C313" s="4"/>
       <c r="D313" s="4"/>
     </row>
-    <row r="314" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A314" s="4"/>
       <c r="C314" s="4"/>
       <c r="D314" s="4"/>
     </row>
-    <row r="315" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A315" s="4"/>
       <c r="C315" s="4"/>
       <c r="D315" s="4"/>
     </row>
-    <row r="316" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A316" s="4"/>
       <c r="C316" s="4"/>
       <c r="D316" s="4"/>
     </row>
-    <row r="317" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A317" s="4"/>
       <c r="C317" s="4"/>
       <c r="D317" s="4"/>
     </row>
-    <row r="318" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A318" s="4"/>
       <c r="C318" s="4"/>
       <c r="D318" s="4"/>
     </row>
-    <row r="319" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A319" s="4"/>
       <c r="C319" s="4"/>
       <c r="D319" s="4"/>
     </row>
-    <row r="320" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A320" s="4"/>
       <c r="C320" s="4"/>
       <c r="D320" s="4"/>
     </row>
-    <row r="321" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A321" s="4"/>
       <c r="C321" s="4"/>
       <c r="D321" s="4"/>
     </row>
-    <row r="322" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A322" s="4"/>
       <c r="C322" s="4"/>
       <c r="D322" s="4"/>
     </row>
-    <row r="323" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A323" s="4"/>
       <c r="C323" s="4"/>
       <c r="D323" s="4"/>
     </row>
-    <row r="324" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A324" s="4"/>
       <c r="C324" s="4"/>
       <c r="D324" s="4"/>
     </row>
-    <row r="325" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A325" s="4"/>
       <c r="C325" s="4"/>
       <c r="D325" s="4"/>
     </row>
-    <row r="326" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A326" s="4"/>
       <c r="C326" s="4"/>
       <c r="D326" s="4"/>
     </row>
-    <row r="327" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A327" s="4"/>
       <c r="C327" s="4"/>
       <c r="D327" s="4"/>
     </row>
-    <row r="328" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A328" s="4"/>
       <c r="C328" s="4"/>
       <c r="D328" s="4"/>
     </row>
-    <row r="329" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A329" s="4"/>
       <c r="C329" s="4"/>
       <c r="D329" s="4"/>
     </row>
-    <row r="330" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A330" s="4"/>
       <c r="C330" s="4"/>
       <c r="D330" s="4"/>
     </row>
-    <row r="331" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A331" s="4"/>
       <c r="C331" s="4"/>
       <c r="D331" s="4"/>
     </row>
-    <row r="332" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A332" s="4"/>
       <c r="C332" s="4"/>
       <c r="D332" s="4"/>
     </row>
-    <row r="333" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A333" s="4"/>
       <c r="C333" s="4"/>
       <c r="D333" s="4"/>
     </row>
-    <row r="334" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A334" s="4"/>
       <c r="C334" s="4"/>
       <c r="D334" s="4"/>
     </row>
-    <row r="335" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A335" s="4"/>
       <c r="C335" s="4"/>
       <c r="D335" s="4"/>
     </row>
-    <row r="336" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A336" s="4"/>
       <c r="C336" s="4"/>
       <c r="D336" s="4"/>
     </row>
-    <row r="337" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A337" s="4"/>
       <c r="C337" s="4"/>
       <c r="D337" s="4"/>
     </row>
-    <row r="338" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A338" s="4"/>
       <c r="C338" s="4"/>
       <c r="D338" s="4"/>
     </row>
-    <row r="339" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A339" s="4"/>
       <c r="C339" s="4"/>
       <c r="D339" s="4"/>
     </row>
-    <row r="340" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A340" s="4"/>
       <c r="C340" s="4"/>
       <c r="D340" s="4"/>
     </row>
-    <row r="341" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A341" s="4"/>
       <c r="C341" s="4"/>
       <c r="D341" s="4"/>
     </row>
-    <row r="342" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A342" s="4"/>
       <c r="C342" s="4"/>
       <c r="D342" s="4"/>
     </row>
-    <row r="343" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A343" s="4"/>
       <c r="C343" s="4"/>
       <c r="D343" s="4"/>
     </row>
-    <row r="344" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A344" s="4"/>
       <c r="C344" s="4"/>
       <c r="D344" s="4"/>
     </row>
-    <row r="345" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A345" s="4"/>
       <c r="C345" s="4"/>
       <c r="D345" s="4"/>
     </row>
-    <row r="346" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A346" s="4"/>
       <c r="C346" s="4"/>
       <c r="D346" s="4"/>
     </row>
-    <row r="347" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A347" s="4"/>
       <c r="C347" s="4"/>
       <c r="D347" s="4"/>
     </row>
-    <row r="348" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A348" s="4"/>
       <c r="C348" s="4"/>
       <c r="D348" s="4"/>
     </row>
-    <row r="349" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A349" s="4"/>
       <c r="C349" s="4"/>
       <c r="D349" s="4"/>
     </row>
-    <row r="350" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A350" s="4"/>
       <c r="C350" s="4"/>
       <c r="D350" s="4"/>
     </row>
-    <row r="351" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A351" s="4"/>
       <c r="C351" s="4"/>
       <c r="D351" s="4"/>
     </row>
-    <row r="352" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A352" s="4"/>
       <c r="C352" s="4"/>
       <c r="D352" s="4"/>
     </row>
-    <row r="353" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A353" s="4"/>
       <c r="C353" s="4"/>
       <c r="D353" s="4"/>
     </row>
-    <row r="354" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A354" s="4"/>
       <c r="C354" s="4"/>
       <c r="D354" s="4"/>
     </row>
-    <row r="355" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A355" s="4"/>
       <c r="C355" s="4"/>
       <c r="D355" s="4"/>
     </row>
-    <row r="356" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A356" s="4"/>
       <c r="C356" s="4"/>
       <c r="D356" s="4"/>
     </row>
-    <row r="357" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A357" s="4"/>
       <c r="C357" s="4"/>
       <c r="D357" s="4"/>
     </row>
-    <row r="358" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A358" s="4"/>
       <c r="C358" s="4"/>
       <c r="D358" s="4"/>
     </row>
-    <row r="359" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A359" s="4"/>
       <c r="C359" s="4"/>
       <c r="D359" s="4"/>
     </row>
-    <row r="360" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A360" s="4"/>
       <c r="C360" s="4"/>
       <c r="D360" s="4"/>
     </row>
-    <row r="361" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A361" s="4"/>
       <c r="C361" s="4"/>
       <c r="D361" s="4"/>
     </row>
-    <row r="362" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A362" s="4"/>
       <c r="C362" s="4"/>
       <c r="D362" s="4"/>
     </row>
-    <row r="363" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A363" s="4"/>
       <c r="C363" s="4"/>
       <c r="D363" s="4"/>
     </row>
-    <row r="364" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A364" s="4"/>
       <c r="C364" s="4"/>
       <c r="D364" s="4"/>
     </row>
-    <row r="365" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A365" s="4"/>
       <c r="C365" s="4"/>
       <c r="D365" s="4"/>
     </row>
-    <row r="366" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A366" s="4"/>
       <c r="C366" s="4"/>
       <c r="D366" s="4"/>
     </row>
-    <row r="367" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A367" s="4"/>
       <c r="C367" s="4"/>
       <c r="D367" s="4"/>
     </row>
-    <row r="368" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A368" s="4"/>
       <c r="C368" s="4"/>
       <c r="D368" s="4"/>
     </row>
-    <row r="369" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A369" s="4"/>
       <c r="C369" s="4"/>
       <c r="D369" s="4"/>
     </row>
-    <row r="370" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A370" s="4"/>
       <c r="C370" s="4"/>
       <c r="D370" s="4"/>
     </row>
-    <row r="371" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A371" s="4"/>
       <c r="C371" s="4"/>
       <c r="D371" s="4"/>
     </row>
-    <row r="372" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A372" s="4"/>
       <c r="C372" s="4"/>
       <c r="D372" s="4"/>
     </row>
-    <row r="373" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A373" s="4"/>
       <c r="C373" s="4"/>
       <c r="D373" s="4"/>
     </row>
-    <row r="374" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A374" s="4"/>
       <c r="C374" s="4"/>
       <c r="D374" s="4"/>
     </row>
-    <row r="375" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A375" s="4"/>
       <c r="C375" s="4"/>
       <c r="D375" s="4"/>
     </row>
-    <row r="376" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A376" s="4"/>
       <c r="C376" s="4"/>
       <c r="D376" s="4"/>
     </row>
-    <row r="377" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A377" s="4"/>
       <c r="C377" s="4"/>
       <c r="D377" s="4"/>
     </row>
-    <row r="378" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A378" s="4"/>
       <c r="C378" s="4"/>
       <c r="D378" s="4"/>
     </row>
-    <row r="379" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A379" s="4"/>
       <c r="C379" s="4"/>
       <c r="D379" s="4"/>
     </row>
-    <row r="380" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A380" s="4"/>
       <c r="C380" s="4"/>
       <c r="D380" s="4"/>
     </row>
-    <row r="381" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A381" s="4"/>
       <c r="C381" s="4"/>
       <c r="D381" s="4"/>
     </row>
-    <row r="382" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A382" s="4"/>
       <c r="C382" s="4"/>
       <c r="D382" s="4"/>
     </row>
-    <row r="383" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A383" s="4"/>
       <c r="C383" s="4"/>
       <c r="D383" s="4"/>
     </row>
-    <row r="384" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A384" s="4"/>
       <c r="C384" s="4"/>
       <c r="D384" s="4"/>
     </row>
-    <row r="385" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A385" s="4"/>
       <c r="C385" s="4"/>
       <c r="D385" s="4"/>
     </row>
-    <row r="386" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A386" s="4"/>
       <c r="C386" s="4"/>
       <c r="D386" s="4"/>
     </row>
-    <row r="387" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A387" s="4"/>
       <c r="C387" s="4"/>
       <c r="D387" s="4"/>
     </row>
-    <row r="388" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A388" s="4"/>
       <c r="C388" s="4"/>
       <c r="D388" s="4"/>
     </row>
-    <row r="389" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A389" s="4"/>
       <c r="C389" s="4"/>
       <c r="D389" s="4"/>
     </row>
-    <row r="390" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A390" s="4"/>
       <c r="C390" s="4"/>
       <c r="D390" s="4"/>
     </row>
-    <row r="391" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A391" s="4"/>
       <c r="C391" s="4"/>
       <c r="D391" s="4"/>
     </row>
-    <row r="392" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A392" s="4"/>
       <c r="C392" s="4"/>
       <c r="D392" s="4"/>
     </row>
-    <row r="393" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A393" s="4"/>
       <c r="C393" s="4"/>
       <c r="D393" s="4"/>
     </row>
-    <row r="394" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A394" s="4"/>
       <c r="C394" s="4"/>
       <c r="D394" s="4"/>
     </row>
-    <row r="395" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A395" s="4"/>
       <c r="C395" s="4"/>
       <c r="D395" s="4"/>
     </row>
-    <row r="396" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A396" s="4"/>
       <c r="C396" s="4"/>
       <c r="D396" s="4"/>
     </row>
-    <row r="397" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A397" s="4"/>
       <c r="C397" s="4"/>
       <c r="D397" s="4"/>
     </row>
-    <row r="398" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A398" s="4"/>
       <c r="C398" s="4"/>
       <c r="D398" s="4"/>
     </row>
-    <row r="399" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A399" s="4"/>
       <c r="C399" s="4"/>
       <c r="D399" s="4"/>
     </row>
-    <row r="400" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A400" s="4"/>
       <c r="C400" s="4"/>
       <c r="D400" s="4"/>
     </row>
-    <row r="401" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A401" s="4"/>
       <c r="C401" s="4"/>
       <c r="D401" s="4"/>
     </row>
-    <row r="402" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A402" s="4"/>
       <c r="C402" s="4"/>
       <c r="D402" s="4"/>
     </row>
-    <row r="403" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A403" s="4"/>
       <c r="C403" s="4"/>
       <c r="D403" s="4"/>
     </row>
-    <row r="404" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A404" s="4"/>
       <c r="C404" s="4"/>
       <c r="D404" s="4"/>
     </row>
-    <row r="405" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A405" s="4"/>
       <c r="C405" s="4"/>
       <c r="D405" s="4"/>
     </row>
-    <row r="406" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A406" s="4"/>
       <c r="C406" s="4"/>
       <c r="D406" s="4"/>
     </row>
-    <row r="407" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A407" s="4"/>
       <c r="C407" s="4"/>
       <c r="D407" s="4"/>
     </row>
-    <row r="408" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A408" s="4"/>
       <c r="C408" s="4"/>
       <c r="D408" s="4"/>
     </row>
-    <row r="409" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A409" s="4"/>
       <c r="C409" s="4"/>
       <c r="D409" s="4"/>
     </row>
-    <row r="410" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A410" s="4"/>
       <c r="C410" s="4"/>
       <c r="D410" s="4"/>
     </row>
-    <row r="411" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A411" s="4"/>
       <c r="C411" s="4"/>
       <c r="D411" s="4"/>
     </row>
-    <row r="412" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A412" s="4"/>
       <c r="C412" s="4"/>
       <c r="D412" s="4"/>
     </row>
-    <row r="413" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A413" s="4"/>
       <c r="C413" s="4"/>
       <c r="D413" s="4"/>
     </row>
-    <row r="414" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A414" s="4"/>
       <c r="C414" s="4"/>
       <c r="D414" s="4"/>
     </row>
-    <row r="415" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A415" s="4"/>
       <c r="C415" s="4"/>
       <c r="D415" s="4"/>
     </row>
-    <row r="416" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A416" s="4"/>
       <c r="C416" s="4"/>
       <c r="D416" s="4"/>
     </row>
-    <row r="417" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A417" s="4"/>
       <c r="C417" s="4"/>
       <c r="D417" s="4"/>
     </row>
-    <row r="418" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A418" s="4"/>
       <c r="C418" s="4"/>
       <c r="D418" s="4"/>
     </row>
-    <row r="419" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A419" s="4"/>
       <c r="C419" s="4"/>
       <c r="D419" s="4"/>
     </row>
-    <row r="420" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A420" s="4"/>
       <c r="C420" s="4"/>
       <c r="D420" s="4"/>
     </row>
-    <row r="421" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A421" s="4"/>
       <c r="C421" s="4"/>
       <c r="D421" s="4"/>

</xml_diff>